<commit_message>
ci: add standalone Selenium E2E Web 300 test workflow and update reports
</commit_message>
<xml_diff>
--- a/selenium-tests/Selenium_Web_E2E_300_Final_Report.xlsx
+++ b/selenium-tests/Selenium_Web_E2E_300_Final_Report.xlsx
@@ -563,7 +563,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Comprehensive 300 Test Cases Verification Report | 100% Pass Rate | Generated: 2026-08-09 22:34:44</t>
+          <t>Comprehensive 300 Test Cases Verification Report | 100% Pass Rate | Generated: 2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="J35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="J41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="J45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3529,7 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4229,7 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="J65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="J67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="J75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="J77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5029,7 +5029,7 @@
       </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J84" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="J85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="J86" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="J87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="J88" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5579,7 @@
       </c>
       <c r="J89" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="J91" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="J92" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5779,7 @@
       </c>
       <c r="J93" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
       </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="J95" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="J96" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="J97" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="J98" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="J99" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="J101" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="J102" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="J103" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="J104" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="J105" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="J106" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="J107" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="J108" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="J109" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="J110" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="J111" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="J112" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6779,7 @@
       </c>
       <c r="J113" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="J114" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="J115" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="J116" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="J117" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="J118" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       </c>
       <c r="J119" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7129,7 +7129,7 @@
       </c>
       <c r="J120" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="J121" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="J123" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="J124" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7379,7 @@
       </c>
       <c r="J125" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="J126" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="J127" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="J128" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7579,7 +7579,7 @@
       </c>
       <c r="J129" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7629,7 +7629,7 @@
       </c>
       <c r="J130" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="J131" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7729,7 @@
       </c>
       <c r="J132" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7779,7 +7779,7 @@
       </c>
       <c r="J133" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="J134" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7879,7 @@
       </c>
       <c r="J135" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="J136" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="J137" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="J138" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="J139" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8129,7 +8129,7 @@
       </c>
       <c r="J140" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="J141" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="J142" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="J143" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="J144" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="J145" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="J146" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="J147" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="J148" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8579,7 @@
       </c>
       <c r="J149" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8629,7 @@
       </c>
       <c r="J150" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="J151" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8729,7 +8729,7 @@
       </c>
       <c r="J152" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="J153" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="J154" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8879,7 +8879,7 @@
       </c>
       <c r="J155" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="J156" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -8979,7 +8979,7 @@
       </c>
       <c r="J157" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9029,7 @@
       </c>
       <c r="J158" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="J159" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="J160" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="J161" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="J162" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="J163" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="J164" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9379,7 +9379,7 @@
       </c>
       <c r="J165" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9429,7 +9429,7 @@
       </c>
       <c r="J166" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9479,7 +9479,7 @@
       </c>
       <c r="J167" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="J168" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9579,7 @@
       </c>
       <c r="J169" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9629,7 +9629,7 @@
       </c>
       <c r="J170" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9679,7 +9679,7 @@
       </c>
       <c r="J171" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="J172" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9779,7 @@
       </c>
       <c r="J173" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="J174" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="J175" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9929,7 +9929,7 @@
       </c>
       <c r="J176" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -9979,7 +9979,7 @@
       </c>
       <c r="J177" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="J178" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10079,7 +10079,7 @@
       </c>
       <c r="J179" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10129,7 @@
       </c>
       <c r="J180" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="J181" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10229,7 @@
       </c>
       <c r="J182" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10279,7 +10279,7 @@
       </c>
       <c r="J183" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10329,7 +10329,7 @@
       </c>
       <c r="J184" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10379,7 +10379,7 @@
       </c>
       <c r="J185" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10429,7 +10429,7 @@
       </c>
       <c r="J186" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10479,7 +10479,7 @@
       </c>
       <c r="J187" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="J188" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10579,7 +10579,7 @@
       </c>
       <c r="J189" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="J190" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10679,7 +10679,7 @@
       </c>
       <c r="J191" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10729,7 +10729,7 @@
       </c>
       <c r="J192" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="J193" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10829,7 +10829,7 @@
       </c>
       <c r="J194" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10879,7 +10879,7 @@
       </c>
       <c r="J195" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="J196" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -10979,7 +10979,7 @@
       </c>
       <c r="J197" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="J198" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="J199" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11129,7 +11129,7 @@
       </c>
       <c r="J200" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="J201" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="J202" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="J203" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11329,7 +11329,7 @@
       </c>
       <c r="J204" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="J205" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11429,7 @@
       </c>
       <c r="J206" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="J207" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11529,7 +11529,7 @@
       </c>
       <c r="J208" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11579,7 +11579,7 @@
       </c>
       <c r="J209" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11629,7 +11629,7 @@
       </c>
       <c r="J210" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="J211" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="J212" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="J213" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="J214" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="J215" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11929,7 +11929,7 @@
       </c>
       <c r="J216" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11979,7 @@
       </c>
       <c r="J217" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="J218" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12079,7 +12079,7 @@
       </c>
       <c r="J219" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12129,7 +12129,7 @@
       </c>
       <c r="J220" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12179,7 +12179,7 @@
       </c>
       <c r="J221" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12229,7 +12229,7 @@
       </c>
       <c r="J222" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12279,7 +12279,7 @@
       </c>
       <c r="J223" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12329,7 +12329,7 @@
       </c>
       <c r="J224" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12379,7 +12379,7 @@
       </c>
       <c r="J225" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="J226" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="J227" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12529,7 +12529,7 @@
       </c>
       <c r="J228" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12579,7 @@
       </c>
       <c r="J229" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12629,7 +12629,7 @@
       </c>
       <c r="J230" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="J231" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12729,7 +12729,7 @@
       </c>
       <c r="J232" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="J233" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="J234" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12879,7 +12879,7 @@
       </c>
       <c r="J235" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12929,7 +12929,7 @@
       </c>
       <c r="J236" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -12979,7 +12979,7 @@
       </c>
       <c r="J237" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="J238" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13079,7 +13079,7 @@
       </c>
       <c r="J239" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13129,7 @@
       </c>
       <c r="J240" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13179,7 +13179,7 @@
       </c>
       <c r="J241" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13229,7 +13229,7 @@
       </c>
       <c r="J242" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13279,7 +13279,7 @@
       </c>
       <c r="J243" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13329,7 +13329,7 @@
       </c>
       <c r="J244" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13379,7 +13379,7 @@
       </c>
       <c r="J245" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13429,7 +13429,7 @@
       </c>
       <c r="J246" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13479,7 +13479,7 @@
       </c>
       <c r="J247" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13529,7 +13529,7 @@
       </c>
       <c r="J248" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13579,7 @@
       </c>
       <c r="J249" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13629,7 +13629,7 @@
       </c>
       <c r="J250" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13679,7 +13679,7 @@
       </c>
       <c r="J251" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13729,7 +13729,7 @@
       </c>
       <c r="J252" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13779,7 +13779,7 @@
       </c>
       <c r="J253" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13829,7 +13829,7 @@
       </c>
       <c r="J254" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="J255" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13929,7 +13929,7 @@
       </c>
       <c r="J256" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -13979,7 +13979,7 @@
       </c>
       <c r="J257" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14029,7 +14029,7 @@
       </c>
       <c r="J258" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="J259" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14129,7 +14129,7 @@
       </c>
       <c r="J260" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14179,7 +14179,7 @@
       </c>
       <c r="J261" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14229,7 +14229,7 @@
       </c>
       <c r="J262" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14279,7 +14279,7 @@
       </c>
       <c r="J263" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14329,7 +14329,7 @@
       </c>
       <c r="J264" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14379,7 @@
       </c>
       <c r="J265" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14429,7 +14429,7 @@
       </c>
       <c r="J266" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14479,7 +14479,7 @@
       </c>
       <c r="J267" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14529,7 +14529,7 @@
       </c>
       <c r="J268" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14579,7 +14579,7 @@
       </c>
       <c r="J269" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
       </c>
       <c r="J270" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14679,7 +14679,7 @@
       </c>
       <c r="J271" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14729,7 @@
       </c>
       <c r="J272" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14779,7 @@
       </c>
       <c r="J273" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14829,7 +14829,7 @@
       </c>
       <c r="J274" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14879,7 +14879,7 @@
       </c>
       <c r="J275" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14929,7 +14929,7 @@
       </c>
       <c r="J276" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -14979,7 +14979,7 @@
       </c>
       <c r="J277" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15029,7 +15029,7 @@
       </c>
       <c r="J278" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15079,7 +15079,7 @@
       </c>
       <c r="J279" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15129,7 +15129,7 @@
       </c>
       <c r="J280" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15179,7 +15179,7 @@
       </c>
       <c r="J281" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15229,7 +15229,7 @@
       </c>
       <c r="J282" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="J283" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
       </c>
       <c r="J284" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="J285" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15429,7 +15429,7 @@
       </c>
       <c r="J286" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15479,7 +15479,7 @@
       </c>
       <c r="J287" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15529,7 +15529,7 @@
       </c>
       <c r="J288" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15579,7 +15579,7 @@
       </c>
       <c r="J289" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15629,7 +15629,7 @@
       </c>
       <c r="J290" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="J291" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15729,7 +15729,7 @@
       </c>
       <c r="J292" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15779,7 +15779,7 @@
       </c>
       <c r="J293" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15829,7 +15829,7 @@
       </c>
       <c r="J294" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15879,7 +15879,7 @@
       </c>
       <c r="J295" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="J296" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -15979,7 +15979,7 @@
       </c>
       <c r="J297" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -16029,7 +16029,7 @@
       </c>
       <c r="J298" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -16079,7 +16079,7 @@
       </c>
       <c r="J299" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -16129,7 +16129,7 @@
       </c>
       <c r="J300" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -16179,7 +16179,7 @@
       </c>
       <c r="J301" s="11" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>
@@ -16229,7 +16229,7 @@
       </c>
       <c r="J302" s="7" t="inlineStr">
         <is>
-          <t>2026-08-09 22:34:44</t>
+          <t>2026-08-10 13:52:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: update 300 test cases Excel and CSV report binaries
</commit_message>
<xml_diff>
--- a/selenium-tests/Selenium_Web_E2E_300_Final_Report.xlsx
+++ b/selenium-tests/Selenium_Web_E2E_300_Final_Report.xlsx
@@ -563,7 +563,7 @@
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Comprehensive 300 Test Cases Verification Report | 100% Pass Rate | Generated: 2026-08-10 13:52:57</t>
+          <t>Comprehensive 300 Test Cases Verification Report | 100% Pass Rate | Generated: 2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="J4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="J6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1579,7 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1679,7 +1679,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1729,7 +1729,7 @@
       </c>
       <c r="J12" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
       </c>
       <c r="J14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1879,7 +1879,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1929,7 @@
       </c>
       <c r="J16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -1979,7 +1979,7 @@
       </c>
       <c r="J17" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="J18" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="J19" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="J20" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2179,7 @@
       </c>
       <c r="J21" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
       </c>
       <c r="J22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="J23" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2329,7 @@
       </c>
       <c r="J24" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="J25" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="J26" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2479,7 +2479,7 @@
       </c>
       <c r="J27" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2529,7 +2529,7 @@
       </c>
       <c r="J28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="J29" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="J30" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J31" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2729,7 +2729,7 @@
       </c>
       <c r="J32" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="J34" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2879,7 @@
       </c>
       <c r="J35" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="J36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="J38" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="J39" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3129,7 +3129,7 @@
       </c>
       <c r="J40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3179,7 @@
       </c>
       <c r="J41" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3229,7 +3229,7 @@
       </c>
       <c r="J42" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3279,7 +3279,7 @@
       </c>
       <c r="J43" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3329,7 +3329,7 @@
       </c>
       <c r="J44" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3379,7 +3379,7 @@
       </c>
       <c r="J45" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3429,7 @@
       </c>
       <c r="J46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="J47" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3529,7 +3529,7 @@
       </c>
       <c r="J48" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3579,7 +3579,7 @@
       </c>
       <c r="J49" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3629,7 @@
       </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="J51" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3779,7 @@
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3829,7 +3829,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="J55" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3929,7 +3929,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -3979,7 +3979,7 @@
       </c>
       <c r="J57" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="J58" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4079,7 @@
       </c>
       <c r="J59" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4129,7 +4129,7 @@
       </c>
       <c r="J60" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4179,7 +4179,7 @@
       </c>
       <c r="J61" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4229,7 @@
       </c>
       <c r="J62" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4279,7 +4279,7 @@
       </c>
       <c r="J63" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="J64" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4379,7 @@
       </c>
       <c r="J65" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4429,7 +4429,7 @@
       </c>
       <c r="J66" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="J67" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4529,7 +4529,7 @@
       </c>
       <c r="J68" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="J69" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="J70" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="J71" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4729,7 @@
       </c>
       <c r="J72" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4779,7 +4779,7 @@
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="J74" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="J75" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4929,7 +4929,7 @@
       </c>
       <c r="J76" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="J77" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5029,7 +5029,7 @@
       </c>
       <c r="J78" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5079,7 +5079,7 @@
       </c>
       <c r="J79" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5129,7 +5129,7 @@
       </c>
       <c r="J80" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="J81" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="J82" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5279,7 +5279,7 @@
       </c>
       <c r="J83" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5329,7 +5329,7 @@
       </c>
       <c r="J84" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5379,7 +5379,7 @@
       </c>
       <c r="J85" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5429,7 @@
       </c>
       <c r="J86" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5479,7 +5479,7 @@
       </c>
       <c r="J87" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5529,7 +5529,7 @@
       </c>
       <c r="J88" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5579,7 @@
       </c>
       <c r="J89" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="J90" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5679,7 +5679,7 @@
       </c>
       <c r="J91" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5729,7 +5729,7 @@
       </c>
       <c r="J92" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5779,7 +5779,7 @@
       </c>
       <c r="J93" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
       </c>
       <c r="J94" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5879,7 +5879,7 @@
       </c>
       <c r="J95" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5929,7 @@
       </c>
       <c r="J96" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -5979,7 +5979,7 @@
       </c>
       <c r="J97" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="J98" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6079,7 +6079,7 @@
       </c>
       <c r="J99" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="J100" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6179,7 +6179,7 @@
       </c>
       <c r="J101" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6229,7 +6229,7 @@
       </c>
       <c r="J102" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="J103" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6329,7 +6329,7 @@
       </c>
       <c r="J104" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6379,7 @@
       </c>
       <c r="J105" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="J106" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6479,7 @@
       </c>
       <c r="J107" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="J108" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="J109" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="J110" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       </c>
       <c r="J111" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="J112" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6779,7 +6779,7 @@
       </c>
       <c r="J113" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6829,7 +6829,7 @@
       </c>
       <c r="J114" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="J115" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6929,7 +6929,7 @@
       </c>
       <c r="J116" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -6979,7 +6979,7 @@
       </c>
       <c r="J117" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="J118" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       </c>
       <c r="J119" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7129,7 +7129,7 @@
       </c>
       <c r="J120" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="J121" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7229,7 +7229,7 @@
       </c>
       <c r="J122" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7279,7 +7279,7 @@
       </c>
       <c r="J123" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="J124" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7379,7 @@
       </c>
       <c r="J125" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7429,7 +7429,7 @@
       </c>
       <c r="J126" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="J127" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7529,7 +7529,7 @@
       </c>
       <c r="J128" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7579,7 +7579,7 @@
       </c>
       <c r="J129" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7629,7 +7629,7 @@
       </c>
       <c r="J130" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="J131" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7729,7 @@
       </c>
       <c r="J132" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7779,7 +7779,7 @@
       </c>
       <c r="J133" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7829,7 +7829,7 @@
       </c>
       <c r="J134" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7879,7 +7879,7 @@
       </c>
       <c r="J135" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="J136" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -7979,7 +7979,7 @@
       </c>
       <c r="J137" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="J138" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="J139" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8129,7 +8129,7 @@
       </c>
       <c r="J140" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8179,7 +8179,7 @@
       </c>
       <c r="J141" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="J142" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8279,7 +8279,7 @@
       </c>
       <c r="J143" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8329,7 +8329,7 @@
       </c>
       <c r="J144" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="J145" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8429,7 +8429,7 @@
       </c>
       <c r="J146" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8479,7 +8479,7 @@
       </c>
       <c r="J147" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="J148" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8579,7 @@
       </c>
       <c r="J149" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8629,7 +8629,7 @@
       </c>
       <c r="J150" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="J151" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8729,7 +8729,7 @@
       </c>
       <c r="J152" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8779,7 +8779,7 @@
       </c>
       <c r="J153" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="J154" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8879,7 +8879,7 @@
       </c>
       <c r="J155" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8929,7 +8929,7 @@
       </c>
       <c r="J156" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -8979,7 +8979,7 @@
       </c>
       <c r="J157" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9029,7 +9029,7 @@
       </c>
       <c r="J158" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9079,7 @@
       </c>
       <c r="J159" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="J160" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9179,7 +9179,7 @@
       </c>
       <c r="J161" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9229,7 +9229,7 @@
       </c>
       <c r="J162" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="J163" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9329,7 +9329,7 @@
       </c>
       <c r="J164" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9379,7 +9379,7 @@
       </c>
       <c r="J165" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9429,7 +9429,7 @@
       </c>
       <c r="J166" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9479,7 +9479,7 @@
       </c>
       <c r="J167" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9529,7 +9529,7 @@
       </c>
       <c r="J168" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9579,7 @@
       </c>
       <c r="J169" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9629,7 +9629,7 @@
       </c>
       <c r="J170" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9679,7 +9679,7 @@
       </c>
       <c r="J171" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9729,7 @@
       </c>
       <c r="J172" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9779,7 +9779,7 @@
       </c>
       <c r="J173" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9829,7 +9829,7 @@
       </c>
       <c r="J174" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9879,7 +9879,7 @@
       </c>
       <c r="J175" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9929,7 +9929,7 @@
       </c>
       <c r="J176" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -9979,7 +9979,7 @@
       </c>
       <c r="J177" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10029,7 +10029,7 @@
       </c>
       <c r="J178" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10079,7 +10079,7 @@
       </c>
       <c r="J179" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10129,7 @@
       </c>
       <c r="J180" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10179,7 +10179,7 @@
       </c>
       <c r="J181" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10229,7 +10229,7 @@
       </c>
       <c r="J182" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10279,7 +10279,7 @@
       </c>
       <c r="J183" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10329,7 +10329,7 @@
       </c>
       <c r="J184" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10379,7 +10379,7 @@
       </c>
       <c r="J185" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10429,7 +10429,7 @@
       </c>
       <c r="J186" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10479,7 +10479,7 @@
       </c>
       <c r="J187" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="J188" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10579,7 +10579,7 @@
       </c>
       <c r="J189" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10629,7 +10629,7 @@
       </c>
       <c r="J190" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10679,7 +10679,7 @@
       </c>
       <c r="J191" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10729,7 +10729,7 @@
       </c>
       <c r="J192" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10779,7 +10779,7 @@
       </c>
       <c r="J193" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10829,7 +10829,7 @@
       </c>
       <c r="J194" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10879,7 +10879,7 @@
       </c>
       <c r="J195" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10929,7 +10929,7 @@
       </c>
       <c r="J196" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -10979,7 +10979,7 @@
       </c>
       <c r="J197" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11029,7 +11029,7 @@
       </c>
       <c r="J198" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11079,7 +11079,7 @@
       </c>
       <c r="J199" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11129,7 +11129,7 @@
       </c>
       <c r="J200" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11179,7 +11179,7 @@
       </c>
       <c r="J201" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11229,7 +11229,7 @@
       </c>
       <c r="J202" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11279,7 +11279,7 @@
       </c>
       <c r="J203" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11329,7 +11329,7 @@
       </c>
       <c r="J204" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="J205" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11429,7 +11429,7 @@
       </c>
       <c r="J206" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11479,7 +11479,7 @@
       </c>
       <c r="J207" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11529,7 +11529,7 @@
       </c>
       <c r="J208" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11579,7 +11579,7 @@
       </c>
       <c r="J209" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11629,7 +11629,7 @@
       </c>
       <c r="J210" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11679,7 +11679,7 @@
       </c>
       <c r="J211" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11729,7 +11729,7 @@
       </c>
       <c r="J212" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="J213" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="J214" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11879,7 +11879,7 @@
       </c>
       <c r="J215" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11929,7 +11929,7 @@
       </c>
       <c r="J216" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11979,7 @@
       </c>
       <c r="J217" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12029,7 +12029,7 @@
       </c>
       <c r="J218" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12079,7 +12079,7 @@
       </c>
       <c r="J219" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12129,7 +12129,7 @@
       </c>
       <c r="J220" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12179,7 +12179,7 @@
       </c>
       <c r="J221" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12229,7 +12229,7 @@
       </c>
       <c r="J222" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12279,7 +12279,7 @@
       </c>
       <c r="J223" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12329,7 +12329,7 @@
       </c>
       <c r="J224" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12379,7 +12379,7 @@
       </c>
       <c r="J225" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12429,7 +12429,7 @@
       </c>
       <c r="J226" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12479,7 +12479,7 @@
       </c>
       <c r="J227" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12529,7 +12529,7 @@
       </c>
       <c r="J228" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12579,7 @@
       </c>
       <c r="J229" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12629,7 +12629,7 @@
       </c>
       <c r="J230" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12679,7 +12679,7 @@
       </c>
       <c r="J231" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12729,7 +12729,7 @@
       </c>
       <c r="J232" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12779,7 +12779,7 @@
       </c>
       <c r="J233" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12829,7 +12829,7 @@
       </c>
       <c r="J234" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12879,7 +12879,7 @@
       </c>
       <c r="J235" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12929,7 +12929,7 @@
       </c>
       <c r="J236" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -12979,7 +12979,7 @@
       </c>
       <c r="J237" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="J238" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13079,7 +13079,7 @@
       </c>
       <c r="J239" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13129,7 +13129,7 @@
       </c>
       <c r="J240" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13179,7 +13179,7 @@
       </c>
       <c r="J241" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13229,7 +13229,7 @@
       </c>
       <c r="J242" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13279,7 +13279,7 @@
       </c>
       <c r="J243" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13329,7 +13329,7 @@
       </c>
       <c r="J244" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13379,7 +13379,7 @@
       </c>
       <c r="J245" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13429,7 +13429,7 @@
       </c>
       <c r="J246" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13479,7 +13479,7 @@
       </c>
       <c r="J247" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13529,7 +13529,7 @@
       </c>
       <c r="J248" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13579,7 +13579,7 @@
       </c>
       <c r="J249" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13629,7 +13629,7 @@
       </c>
       <c r="J250" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13679,7 +13679,7 @@
       </c>
       <c r="J251" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13729,7 +13729,7 @@
       </c>
       <c r="J252" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13779,7 +13779,7 @@
       </c>
       <c r="J253" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13829,7 +13829,7 @@
       </c>
       <c r="J254" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13879,7 +13879,7 @@
       </c>
       <c r="J255" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13929,7 +13929,7 @@
       </c>
       <c r="J256" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -13979,7 +13979,7 @@
       </c>
       <c r="J257" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14029,7 +14029,7 @@
       </c>
       <c r="J258" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14079,7 +14079,7 @@
       </c>
       <c r="J259" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14129,7 +14129,7 @@
       </c>
       <c r="J260" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14179,7 +14179,7 @@
       </c>
       <c r="J261" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14229,7 +14229,7 @@
       </c>
       <c r="J262" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14279,7 +14279,7 @@
       </c>
       <c r="J263" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14329,7 +14329,7 @@
       </c>
       <c r="J264" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14379,7 @@
       </c>
       <c r="J265" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14429,7 +14429,7 @@
       </c>
       <c r="J266" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14479,7 +14479,7 @@
       </c>
       <c r="J267" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14529,7 +14529,7 @@
       </c>
       <c r="J268" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14579,7 +14579,7 @@
       </c>
       <c r="J269" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
       </c>
       <c r="J270" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14679,7 +14679,7 @@
       </c>
       <c r="J271" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14729,7 +14729,7 @@
       </c>
       <c r="J272" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14779,7 +14779,7 @@
       </c>
       <c r="J273" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14829,7 +14829,7 @@
       </c>
       <c r="J274" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14879,7 +14879,7 @@
       </c>
       <c r="J275" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14929,7 +14929,7 @@
       </c>
       <c r="J276" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -14979,7 +14979,7 @@
       </c>
       <c r="J277" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15029,7 +15029,7 @@
       </c>
       <c r="J278" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15079,7 +15079,7 @@
       </c>
       <c r="J279" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15129,7 +15129,7 @@
       </c>
       <c r="J280" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15179,7 +15179,7 @@
       </c>
       <c r="J281" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15229,7 +15229,7 @@
       </c>
       <c r="J282" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="J283" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
       </c>
       <c r="J284" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="J285" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15429,7 +15429,7 @@
       </c>
       <c r="J286" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15479,7 +15479,7 @@
       </c>
       <c r="J287" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15529,7 +15529,7 @@
       </c>
       <c r="J288" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15579,7 +15579,7 @@
       </c>
       <c r="J289" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15629,7 +15629,7 @@
       </c>
       <c r="J290" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15679,7 +15679,7 @@
       </c>
       <c r="J291" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15729,7 +15729,7 @@
       </c>
       <c r="J292" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15779,7 +15779,7 @@
       </c>
       <c r="J293" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15829,7 +15829,7 @@
       </c>
       <c r="J294" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15879,7 +15879,7 @@
       </c>
       <c r="J295" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15929,7 +15929,7 @@
       </c>
       <c r="J296" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -15979,7 +15979,7 @@
       </c>
       <c r="J297" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -16029,7 +16029,7 @@
       </c>
       <c r="J298" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -16079,7 +16079,7 @@
       </c>
       <c r="J299" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -16129,7 +16129,7 @@
       </c>
       <c r="J300" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -16179,7 +16179,7 @@
       </c>
       <c r="J301" s="11" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>
@@ -16229,7 +16229,7 @@
       </c>
       <c r="J302" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10 13:52:57</t>
+          <t>2026-08-10 14:05:47</t>
         </is>
       </c>
     </row>

</xml_diff>